<commit_message>
docs(diy): one pinout sheet per LCD for xiao-s3-tft and handheld-s3
xiao-s3-tft: ILI9488 3.5in (current) and the ILI9341 3.2in pinout (environment
removed in d5dfbffb8, never verified on hardware).
handheld-s3: ILI9341 2.4in, ILI9341 3.2in, ILI9488 4.0in and the joystick wiring.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/variants/esp32s3/diy/RiV_handheld-s3/RiV_handheld-s3_pinout.xlsx
+++ b/variants/esp32s3/diy/RiV_handheld-s3/RiV_handheld-s3_pinout.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pinout" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="joystick" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ILI9341 2.4in" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ILI9341 3.2in" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ILI9488 4.0in" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="joystick" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -585,7 +587,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>LCD (ILI9341 / ILI9488, same pins)</t>
+          <t>ILI9341 2.4in (LCD)</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -657,234 +659,249 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>LCD_MISO/SDO</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>XPT2046 touch</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Signal</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>T_CS</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C20" s="2" t="n"/>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>T_CS</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
           <t>T_IRQ</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B22" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C21" s="2" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="C22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>SD card</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Signal</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>SD_CS</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B25" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C24" s="2" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="C25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>I2C</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Signal</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>SDA</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>CardKB 0x5F, BMP280</t>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>SDA</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>CardKB 0x5F, BMP280</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>SCL</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B29" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C28" s="2" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="C29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>GPS</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Signal</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>GPS_TX</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>module TX to ESP RX</t>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>GPS_TX</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>module TX to ESP RX</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>GPS_RX</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B33" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>module RX to ESP TX</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>Signal</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>GPIO</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="B34" s="3" t="n"/>
+      <c r="C34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>BOOT</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B36" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C35" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -892,6 +909,952 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RiV_handheld-s3-32in</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Shared SPI bus</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SCK</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>MISO</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>MOSI</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>LoRa RFM95W</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>RESET</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>DIO0</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>IRQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>ILI9341 3.2in (LCD)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>LCD_CS</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>LCD_DC</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>LCD_RST</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>LCD_BL</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>PWM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>LCD_MISO/SDO</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>shared</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>XPT2046 touch</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>T_CS</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>touch rotation 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>T_IRQ</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>SD card</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>SD_CS</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>I2C</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>SDA</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>CardKB 0x5F, BMP280</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>SCL</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>GPS</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>GPS_TX</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>module TX to ESP RX</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>GPS_RX</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>module RX to ESP TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n"/>
+      <c r="C34" s="3" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>BOOT</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RiV_handheld-s3-4in</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Shared SPI bus</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SCK</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>MISO</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>MOSI</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>LoRa RFM95W</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>RESET</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>DIO0</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>IRQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>ILI9488 4.0in IPS (LCD)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>LCD_CS</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>LCD_DC</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="C15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>LCD_RST</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>LCD_BL</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>PWM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>LCD_MISO/SDO</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>leave the LCD SDO unwired</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>XPT2046 touch</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>T_CS</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>touch rotation 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>T_IRQ</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>SD card</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n"/>
+      <c r="C23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>SD_CS</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>I2C</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>SDA</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>CardKB 0x5F, BMP280</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>SCL</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>GPS</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>GPS_TX</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>module TX to ESP RX</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>GPS_RX</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>module RX to ESP TX</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n"/>
+      <c r="C34" s="3" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>GPIO</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>BOOT</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs(handheld-s3): show the ILI9488 LCD SDO as not connected in the pinout
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/variants/esp32s3/diy/RiV_handheld-s3/RiV_handheld-s3_pinout.xlsx
+++ b/variants/esp32s3/diy/RiV_handheld-s3/RiV_handheld-s3_pinout.xlsx
@@ -1606,12 +1606,14 @@
           <t>LCD_MISO/SDO</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
-        <v>13</v>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>leave the LCD SDO unwired</t>
+          <t>not connected; it jams the radio</t>
         </is>
       </c>
     </row>

</xml_diff>